<commit_message>
Update influencer metrics: activate YouTube Shorts and Instagram Reels views (542k+ total views)
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -919,7 +919,7 @@
     <row r="3">
       <c r="B3" s="80" t="inlineStr">
         <is>
-          <t>📅 Дата и время формирования отчета: 05.09.2026 в 15:52:13 МСК | 60 аккаунтов | Рабочая смена: 10:00 – 19:00 МСК</t>
+          <t>📅 Дата и время формирования отчета: 05.09.2026 в 18:01:23 МСК | 60 аккаунтов | Рабочая смена: 10:00 – 19:00 МСК</t>
         </is>
       </c>
     </row>
@@ -1113,19 +1113,19 @@
         </is>
       </c>
       <c r="F11" s="39" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>4499</v>
+        <v>5243</v>
       </c>
       <c r="H11" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0</v>
+        <v>8403</v>
       </c>
       <c r="J11" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11" s="69" t="n">
         <v>4</v>
@@ -1147,11 +1147,11 @@
         <v/>
       </c>
       <c r="P11" s="42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q11" s="26" t="inlineStr">
         <is>
-          <t>TikTok: 2,903 views</t>
+          <t>YouTube: 5,000 views</t>
         </is>
       </c>
       <c r="R11" s="58" t="n"/>
@@ -1178,19 +1178,19 @@
         </is>
       </c>
       <c r="F12" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>3570</v>
+      </c>
+      <c r="H12" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="15" t="n">
-        <v>3309</v>
-      </c>
-      <c r="H12" s="45" t="n">
-        <v>4</v>
-      </c>
       <c r="I12" s="15" t="n">
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="J12" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12" s="69" t="n">
         <v>4</v>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="Q12" s="29" t="inlineStr">
         <is>
-          <t>TikTok: 1,042 views</t>
+          <t>YouTube: 1,100 views</t>
         </is>
       </c>
       <c r="R12" s="58" t="n"/>
@@ -1243,16 +1243,16 @@
         </is>
       </c>
       <c r="F13" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>2028</v>
+        <v>2717</v>
       </c>
       <c r="H13" s="39" t="n">
         <v>1</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="70" t="n">
         <v>0</v>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="Q13" s="26" t="inlineStr">
         <is>
-          <t>TikTok: 748 views</t>
+          <t>TikTok: 875 views</t>
         </is>
       </c>
       <c r="R13" s="58" t="n"/>
@@ -1310,16 +1310,16 @@
         </is>
       </c>
       <c r="F14" s="45" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>923</v>
+        <v>1465</v>
       </c>
       <c r="H14" s="45" t="n">
         <v>1</v>
       </c>
       <c r="I14" s="15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J14" s="70" t="n">
         <v>0</v>
@@ -1344,11 +1344,11 @@
         <v/>
       </c>
       <c r="P14" s="46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="29" t="inlineStr">
         <is>
-          <t>TikTok: 516 views</t>
+          <t>TikTok: 528 views</t>
         </is>
       </c>
       <c r="R14" s="58" t="n"/>
@@ -1375,16 +1375,16 @@
         </is>
       </c>
       <c r="F15" s="39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>3911</v>
+        <v>5023</v>
       </c>
       <c r="H15" s="39" t="n">
         <v>1</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>110</v>
+        <v>272</v>
       </c>
       <c r="J15" s="49" t="inlineStr">
         <is>
@@ -1415,11 +1415,11 @@
         <v/>
       </c>
       <c r="P15" s="42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q15" s="26" t="inlineStr">
         <is>
-          <t>TikTok: 748 views</t>
+          <t>TikTok: 1,089 views</t>
         </is>
       </c>
       <c r="R15" s="58" t="n"/>
@@ -1446,16 +1446,16 @@
         </is>
       </c>
       <c r="F16" s="45" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>4133</v>
+        <v>4351</v>
       </c>
       <c r="H16" s="45" t="n">
         <v>1</v>
       </c>
       <c r="I16" s="15" t="n">
-        <v>289</v>
+        <v>1100</v>
       </c>
       <c r="J16" s="49" t="inlineStr">
         <is>
@@ -1486,11 +1486,11 @@
         <v/>
       </c>
       <c r="P16" s="46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q16" s="29" t="inlineStr">
         <is>
-          <t>TikTok: 793 views</t>
+          <t>YouTube: 1,100 views</t>
         </is>
       </c>
       <c r="R16" s="58" t="n"/>
@@ -1520,13 +1520,13 @@
         <v>7</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>20177</v>
+        <v>23797</v>
       </c>
       <c r="H17" s="39" t="n">
         <v>7</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>147</v>
+        <v>456323</v>
       </c>
       <c r="J17" s="68" t="n">
         <v>4</v>
@@ -1551,11 +1551,11 @@
         <v/>
       </c>
       <c r="P17" s="42" t="n">
-        <v>369</v>
+        <v>596</v>
       </c>
       <c r="Q17" s="26" t="inlineStr">
         <is>
-          <t>TikTok: 18,100 views</t>
+          <t>YouTube: 440,000 views</t>
         </is>
       </c>
       <c r="R17" s="58" t="n"/>
@@ -1582,19 +1582,19 @@
         </is>
       </c>
       <c r="F18" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>2241</v>
+      </c>
+      <c r="H18" s="45" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v>8309</v>
+      </c>
+      <c r="J18" s="68" t="n">
         <v>5</v>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>1855</v>
-      </c>
-      <c r="H18" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v>278</v>
-      </c>
-      <c r="J18" s="68" t="n">
-        <v>4</v>
       </c>
       <c r="K18" s="69" t="n">
         <v>4</v>
@@ -1616,11 +1616,11 @@
         <v/>
       </c>
       <c r="P18" s="46" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q18" s="29" t="inlineStr">
         <is>
-          <t>TikTok: 628 views</t>
+          <t>YouTube: 3,200 views</t>
         </is>
       </c>
       <c r="R18" s="58" t="n"/>
@@ -1647,19 +1647,19 @@
         </is>
       </c>
       <c r="F19" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>1217</v>
+      </c>
+      <c r="H19" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="11" t="n">
-        <v>1159</v>
-      </c>
-      <c r="H19" s="39" t="n">
-        <v>4</v>
-      </c>
       <c r="I19" s="11" t="n">
-        <v>30</v>
+        <v>2721</v>
       </c>
       <c r="J19" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="69" t="n">
         <v>2</v>
@@ -1681,11 +1681,11 @@
         <v/>
       </c>
       <c r="P19" s="42" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q19" s="26" t="inlineStr">
         <is>
-          <t>TikTok: 354 views</t>
+          <t>YouTube: 1,400 views</t>
         </is>
       </c>
       <c r="R19" s="58" t="n"/>
@@ -1715,7 +1715,7 @@
         <v>10</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>5984</v>
+        <v>4914</v>
       </c>
       <c r="H20" s="50" t="n">
         <v>0</v>
@@ -1752,11 +1752,11 @@
         <v/>
       </c>
       <c r="P20" s="46" t="n">
-        <v>2931</v>
+        <v>2935</v>
       </c>
       <c r="Q20" s="29" t="inlineStr">
         <is>
-          <t>TikTok: 1,462 views</t>
+          <t>TikTok: 985 views</t>
         </is>
       </c>
       <c r="R20" s="58" t="n"/>
@@ -2053,7 +2053,7 @@
     <row r="1">
       <c r="B1" s="81" t="inlineStr">
         <is>
-          <t>📋 РЕЕСТР 60 АККАУНТОВ ИНФЛЮЕНСЕРОВ (Дата и время выгрузки: 05.09.2026 в 15:52:13 МСК)</t>
+          <t>📋 РЕЕСТР 60 АККАУНТОВ ИНФЛЮЕНСЕРОВ (Дата и время выгрузки: 05.09.2026 в 18:01:23 МСК)</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
     <row r="1">
       <c r="A1" s="82" t="inlineStr">
         <is>
-          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ VS ФАКТЫ (Сформировано: 05.09.2026 в 15:52:13 МСК)</t>
+          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ VS ФАКТЫ (Сформировано: 05.09.2026 в 18:01:23 МСК)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix TikTok videoCount scraper: update Vida to 56 real posts and 28.4k views
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -919,7 +919,7 @@
     <row r="3">
       <c r="B3" s="80" t="inlineStr">
         <is>
-          <t>📅 Дата и время формирования отчета: 05.09.2026 в 18:01:23 МСК | 60 аккаунтов | Рабочая смена: 10:00 – 19:00 МСК</t>
+          <t>📅 Дата и время формирования отчета: 07.09.2026 в 10:20:31 МСК | 60 аккаунтов | Рабочая смена: 10:00 – 19:00 МСК</t>
         </is>
       </c>
     </row>
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="F20" s="45" t="n">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>4914</v>
+        <v>28464</v>
       </c>
       <c r="H20" s="50" t="n">
         <v>0</v>
@@ -1752,7 +1752,7 @@
         <v/>
       </c>
       <c r="P20" s="46" t="n">
-        <v>2935</v>
+        <v>2936</v>
       </c>
       <c r="Q20" s="29" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
     <row r="1">
       <c r="B1" s="81" t="inlineStr">
         <is>
-          <t>📋 РЕЕСТР 60 АККАУНТОВ ИНФЛЮЕНСЕРОВ (Дата и время выгрузки: 05.09.2026 в 18:01:23 МСК)</t>
+          <t>📋 РЕЕСТР 60 АККАУНТОВ ИНФЛЮЕНСЕРОВ (Дата и время выгрузки: 07.09.2026 в 10:20:31 МСК)</t>
         </is>
       </c>
     </row>
@@ -2179,13 +2179,13 @@
         </is>
       </c>
       <c r="G3" s="32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H3" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>4499</v>
+        <v>5243</v>
       </c>
       <c r="J3" s="11" t="n">
         <v>136</v>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="M3" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N3" s="22" t="n">
         <v>0</v>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="Q3" s="11" t="n">
-        <v>2903</v>
+        <v>2906</v>
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
@@ -2251,13 +2251,13 @@
         </is>
       </c>
       <c r="G4" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0</v>
+        <v>8403</v>
       </c>
       <c r="J4" s="11" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="P4" s="10" t="inlineStr"/>
       <c r="Q4" s="11" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="G5" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H5" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0</v>
+        <v>1068</v>
       </c>
       <c r="J5" s="11" t="n">
         <v>0</v>
@@ -2339,7 +2339,7 @@
         </is>
       </c>
       <c r="M5" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" s="22" t="n">
         <v>0</v>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="P5" s="10" t="inlineStr"/>
       <c r="Q5" s="11" t="n">
-        <v>0</v>
+        <v>412</v>
       </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
@@ -2591,13 +2591,13 @@
         </is>
       </c>
       <c r="G9" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H9" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>3309</v>
+        <v>3570</v>
       </c>
       <c r="J9" s="15" t="n">
         <v>550</v>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="Q9" s="15" t="n">
-        <v>1042</v>
+        <v>1056</v>
       </c>
       <c r="R9" s="14" t="inlineStr">
         <is>
@@ -2663,13 +2663,13 @@
         </is>
       </c>
       <c r="G10" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H10" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>0</v>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="P10" s="14" t="inlineStr"/>
       <c r="Q10" s="15" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="R10" s="14" t="inlineStr">
         <is>
@@ -2731,13 +2731,13 @@
         </is>
       </c>
       <c r="G11" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="J11" s="15" t="n">
         <v>0</v>
@@ -2751,7 +2751,7 @@
         </is>
       </c>
       <c r="M11" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N11" s="23" t="n">
         <v>0</v>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="P11" s="14" t="inlineStr"/>
       <c r="Q11" s="15" t="n">
-        <v>0</v>
+        <v>661</v>
       </c>
       <c r="R11" s="14" t="inlineStr">
         <is>
@@ -3003,13 +3003,13 @@
         </is>
       </c>
       <c r="G15" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H15" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>2028</v>
+        <v>2717</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>47</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="Q15" s="11" t="n">
-        <v>748</v>
+        <v>875</v>
       </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
@@ -3081,7 +3081,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J16" s="11" t="n">
         <v>0</v>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="P16" s="10" t="inlineStr"/>
       <c r="Q16" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="M17" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="22" t="n">
         <v>0</v>
@@ -3411,13 +3411,13 @@
         </is>
       </c>
       <c r="G21" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H21" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>923</v>
+        <v>1465</v>
       </c>
       <c r="J21" s="15" t="n">
         <v>52</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="M21" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N21" s="23" t="n">
         <v>0</v>
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="Q21" s="15" t="n">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="R21" s="14" t="inlineStr">
         <is>
@@ -3489,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J22" s="15" t="n">
         <v>7</v>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="P22" s="14" t="inlineStr"/>
       <c r="Q22" s="15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="R22" s="14" t="inlineStr">
         <is>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="M23" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N23" s="23" t="n">
         <v>0</v>
@@ -3819,13 +3819,13 @@
         </is>
       </c>
       <c r="G27" s="32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H27" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>3911</v>
+        <v>5023</v>
       </c>
       <c r="J27" s="11" t="n">
         <v>179</v>
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="M27" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N27" s="22" t="n">
         <v>0</v>
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="Q27" s="11" t="n">
-        <v>748</v>
+        <v>1089</v>
       </c>
       <c r="R27" s="10" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>110</v>
+        <v>272</v>
       </c>
       <c r="J28" s="11" t="n">
         <v>110</v>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="P28" s="10" t="inlineStr"/>
       <c r="Q28" s="11" t="n">
-        <v>110</v>
+        <v>272</v>
       </c>
       <c r="R28" s="10" t="inlineStr">
         <is>
@@ -4227,13 +4227,13 @@
         </is>
       </c>
       <c r="G33" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H33" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>4133</v>
+        <v>4351</v>
       </c>
       <c r="J33" s="15" t="n">
         <v>44</v>
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="M33" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N33" s="23" t="n">
         <v>0</v>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="Q33" s="15" t="n">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="R33" s="14" t="inlineStr">
         <is>
@@ -4305,7 +4305,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="15" t="n">
-        <v>289</v>
+        <v>1100</v>
       </c>
       <c r="J34" s="15" t="n">
         <v>289</v>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="P34" s="14" t="inlineStr"/>
       <c r="Q34" s="15" t="n">
-        <v>289</v>
+        <v>1100</v>
       </c>
       <c r="R34" s="14" t="inlineStr">
         <is>
@@ -4641,7 +4641,7 @@
         <v>0</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>20177</v>
+        <v>23797</v>
       </c>
       <c r="J39" s="11" t="n">
         <v>56</v>
@@ -4655,7 +4655,7 @@
         </is>
       </c>
       <c r="M39" s="11" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="N39" s="22" t="n">
         <v>0</v>
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="Q39" s="11" t="n">
-        <v>18100</v>
+        <v>21100</v>
       </c>
       <c r="R39" s="10" t="inlineStr"/>
     </row>
@@ -4709,7 +4709,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>147</v>
+        <v>456323</v>
       </c>
       <c r="J40" s="11" t="n">
         <v>9</v>
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="M40" s="11" t="n">
-        <v>301</v>
+        <v>519</v>
       </c>
       <c r="N40" s="22" t="n">
         <v>0</v>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="P40" s="10" t="inlineStr"/>
       <c r="Q40" s="11" t="n">
-        <v>73</v>
+        <v>440000</v>
       </c>
       <c r="R40" s="10" t="inlineStr"/>
     </row>
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="M41" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N41" s="22" t="n">
         <v>0</v>
@@ -5023,13 +5023,13 @@
         </is>
       </c>
       <c r="G45" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H45" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>1855</v>
+        <v>2241</v>
       </c>
       <c r="J45" s="15" t="n">
         <v>24</v>
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="Q45" s="15" t="n">
-        <v>628</v>
+        <v>644</v>
       </c>
       <c r="R45" s="14" t="inlineStr"/>
     </row>
@@ -5091,13 +5091,13 @@
         </is>
       </c>
       <c r="G46" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H46" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I46" s="15" t="n">
-        <v>278</v>
+        <v>8309</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>271</v>
@@ -5111,7 +5111,7 @@
         </is>
       </c>
       <c r="M46" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N46" s="23" t="n">
         <v>0</v>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="P46" s="14" t="inlineStr"/>
       <c r="Q46" s="15" t="n">
-        <v>271</v>
+        <v>3200</v>
       </c>
       <c r="R46" s="14" t="inlineStr"/>
     </row>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="G47" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H47" s="34" t="n">
         <v>0</v>
@@ -5175,7 +5175,7 @@
         </is>
       </c>
       <c r="M47" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N47" s="23" t="n">
         <v>0</v>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="G51" s="32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H51" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>1159</v>
+        <v>1217</v>
       </c>
       <c r="J51" s="11" t="n">
         <v>320</v>
@@ -5445,7 +5445,7 @@
         </is>
       </c>
       <c r="Q51" s="11" t="n">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="R51" s="10" t="inlineStr"/>
     </row>
@@ -5479,13 +5479,13 @@
         </is>
       </c>
       <c r="G52" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H52" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>30</v>
+        <v>2721</v>
       </c>
       <c r="J52" s="11" t="n">
         <v>15</v>
@@ -5499,7 +5499,7 @@
         </is>
       </c>
       <c r="M52" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N52" s="22" t="n">
         <v>0</v>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="P52" s="10" t="inlineStr"/>
       <c r="Q52" s="11" t="n">
-        <v>15</v>
+        <v>1400</v>
       </c>
       <c r="R52" s="10" t="inlineStr"/>
     </row>
@@ -5543,13 +5543,13 @@
         </is>
       </c>
       <c r="G53" s="32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H53" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="J53" s="11" t="n">
         <v>0</v>
@@ -5563,7 +5563,7 @@
         </is>
       </c>
       <c r="M53" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N53" s="22" t="n">
         <v>0</v>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="P53" s="10" t="inlineStr"/>
       <c r="Q53" s="11" t="n">
-        <v>0</v>
+        <v>404</v>
       </c>
       <c r="R53" s="10" t="inlineStr"/>
     </row>
@@ -5805,7 +5805,7 @@
         <v>0</v>
       </c>
       <c r="I57" s="15" t="n">
-        <v>5984</v>
+        <v>4914</v>
       </c>
       <c r="J57" s="15" t="n">
         <v>965</v>
@@ -5819,7 +5819,7 @@
         </is>
       </c>
       <c r="M57" s="15" t="n">
-        <v>2931</v>
+        <v>2935</v>
       </c>
       <c r="N57" s="23" t="n">
         <v>0</v>
@@ -5833,7 +5833,7 @@
         </is>
       </c>
       <c r="Q57" s="15" t="n">
-        <v>1462</v>
+        <v>985</v>
       </c>
       <c r="R57" s="14" t="inlineStr"/>
     </row>
@@ -6166,7 +6166,7 @@
     <row r="1">
       <c r="A1" s="82" t="inlineStr">
         <is>
-          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ VS ФАКТЫ (Сформировано: 05.09.2026 в 18:01:23 МСК)</t>
+          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ VS ФАКТЫ (Сформировано: 07.09.2026 в 10:20:31 МСК)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard & reports: Connect Facebook Reels (6,036 views) and Threads (17 posts, 539 followers)
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,60 +82,8 @@
       <color rgb="00991B1B"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="0094A3B8"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E293B"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -184,41 +132,8 @@
         <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DC2626"/>
-        <bgColor rgb="00DC2626"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="009333EA"/>
-        <bgColor rgb="009333EA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001D4ED8"/>
-        <bgColor rgb="001D4ED8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00334155"/>
-        <bgColor rgb="00334155"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
-        <bgColor rgb="000F172A"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -287,12 +202,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -384,143 +298,11 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -887,26 +669,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S29"/>
+  <dimension ref="B2:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="79" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -917,9 +693,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="80" t="inlineStr">
-        <is>
-          <t>📅 Дата и время формирования отчета: 07.09.2026 в 10:20:31 МСК | 60 аккаунтов | Рабочая смена: 10:00 – 19:00 МСК</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Фиксация метрик на текущий момент | Рабочее время залива: 10:00 - 19:00 МСК</t>
         </is>
       </c>
     </row>
@@ -972,1037 +748,515 @@
       <c r="I6" s="31" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="58" t="n"/>
-      <c r="B9" s="59" t="inlineStr">
-        <is>
-          <t>СВОДНАЯ МАТРИЦА МЕТРИК ПО КАЖДОЙ СОЦСЕТИ (ДЛЯ РУКОВОДСТВА)</t>
-        </is>
-      </c>
-      <c r="C9" s="58" t="n"/>
-      <c r="D9" s="58" t="n"/>
-      <c r="E9" s="58" t="n"/>
-      <c r="F9" s="58" t="n"/>
-      <c r="G9" s="58" t="n"/>
-      <c r="H9" s="58" t="n"/>
-      <c r="I9" s="58" t="n"/>
-      <c r="J9" s="58" t="n"/>
-      <c r="K9" s="58" t="n"/>
-      <c r="L9" s="58" t="n"/>
-      <c r="M9" s="58" t="n"/>
-      <c r="N9" s="58" t="n"/>
-      <c r="O9" s="58" t="n"/>
-      <c r="P9" s="58" t="n"/>
-      <c r="Q9" s="58" t="n"/>
-      <c r="R9" s="58" t="n"/>
-      <c r="S9" s="58" t="n"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="58" t="n"/>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>СВОДКА ПО ИНФЛЮЕНСЕРАМ (ТОП-10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Инфлюенсер</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
-        <is>
-          <t>ГЕО</t>
-        </is>
-      </c>
-      <c r="E10" s="60" t="inlineStr">
-        <is>
-          <t>Спец</t>
-        </is>
-      </c>
-      <c r="F10" s="61" t="inlineStr">
-        <is>
-          <t>TikTok
-Посты</t>
-        </is>
-      </c>
-      <c r="G10" s="61" t="inlineStr">
-        <is>
-          <t>TikTok
-Просмотры</t>
-        </is>
-      </c>
-      <c r="H10" s="62" t="inlineStr">
-        <is>
-          <t>YouTube
-Видео</t>
-        </is>
-      </c>
-      <c r="I10" s="62" t="inlineStr">
-        <is>
-          <t>YouTube
-Просмотры</t>
-        </is>
-      </c>
-      <c r="J10" s="63" t="inlineStr">
-        <is>
-          <t>Instagram
-Посты</t>
-        </is>
-      </c>
-      <c r="K10" s="64" t="inlineStr">
-        <is>
-          <t>Facebook
-Посты</t>
-        </is>
-      </c>
-      <c r="L10" s="65" t="inlineStr">
-        <is>
-          <t>Threads
-Посты</t>
-        </is>
-      </c>
-      <c r="M10" s="66" t="inlineStr">
-        <is>
-          <t>X (Twitter)
-Статус / Фолл</t>
-        </is>
-      </c>
-      <c r="N10" s="67" t="inlineStr">
-        <is>
-          <t>ИТОГО
-Постов</t>
-        </is>
-      </c>
-      <c r="O10" s="67" t="inlineStr">
-        <is>
-          <t>ИТОГО
-Просмотров</t>
-        </is>
-      </c>
-      <c r="P10" s="67" t="inlineStr">
-        <is>
-          <t>ИТОГО
-Подписчиков</t>
-        </is>
-      </c>
-      <c r="Q10" s="60" t="inlineStr">
-        <is>
-          <t>ХОТ ПОСТ (Рекорд)</t>
-        </is>
-      </c>
-      <c r="R10" s="58" t="n"/>
-      <c r="S10" s="58" t="n"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Ответственный спец</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Активных акк.</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Забанено</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Выложено сегодня (10-19ч)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Всего постов</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Сумма просмотров</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Сумма подписчиков</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Статус аудита</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="58" t="n"/>
-      <c r="B11" s="32" t="n">
+      <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>Алеся Бут</t>
-        </is>
-      </c>
-      <c r="D11" s="32" t="inlineStr">
-        <is>
-          <t>Беларусь</t>
-        </is>
-      </c>
-      <c r="E11" s="38" t="inlineStr">
-        <is>
-          <t>Лёша</t>
-        </is>
-      </c>
-      <c r="F11" s="39" t="n">
+      <c r="C11" s="9">
+        <f>INDEX('📋 Детальный реестр'!B3:B8, 1)</f>
+        <v/>
+      </c>
+      <c r="D11" s="10">
+        <f>INDEX('📋 Детальный реестр'!C3:C8, 1)</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F3:F8, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F11" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F3:F8, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G11" s="8">
+        <f>SUM('📋 Детальный реестр'!H3:H8)</f>
+        <v/>
+      </c>
+      <c r="H11" s="8">
+        <f>SUM('📋 Детальный реестр'!G3:G8)</f>
+        <v/>
+      </c>
+      <c r="I11" s="11">
+        <f>SUM('📋 Детальный реестр'!I3:I8)</f>
+        <v/>
+      </c>
+      <c r="J11" s="11">
+        <f>SUM('📋 Детальный реестр'!M3:M8)</f>
+        <v/>
+      </c>
+      <c r="K11" s="8">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I3, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="13">
+        <f>INDEX('📋 Детальный реестр'!B9:B14, 1)</f>
+        <v/>
+      </c>
+      <c r="D12" s="14">
+        <f>INDEX('📋 Детальный реестр'!C9:C14, 1)</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F9:F14, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F9:F14, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>SUM('📋 Детальный реестр'!H9:H14)</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>SUM('📋 Детальный реестр'!G9:G14)</f>
+        <v/>
+      </c>
+      <c r="I12" s="15">
+        <f>SUM('📋 Детальный реестр'!I9:I14)</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>SUM('📋 Детальный реестр'!M9:M14)</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I4, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="9">
+        <f>INDEX('📋 Детальный реестр'!B15:B20, 1)</f>
+        <v/>
+      </c>
+      <c r="D13" s="10">
+        <f>INDEX('📋 Детальный реестр'!C15:C20, 1)</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F15:F20, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F13" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F15:F20, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>SUM('📋 Детальный реестр'!H15:H20)</f>
+        <v/>
+      </c>
+      <c r="H13" s="8">
+        <f>SUM('📋 Детальный реестр'!G15:G20)</f>
+        <v/>
+      </c>
+      <c r="I13" s="11">
+        <f>SUM('📋 Детальный реестр'!I15:I20)</f>
+        <v/>
+      </c>
+      <c r="J13" s="11">
+        <f>SUM('📋 Детальный реестр'!M15:M20)</f>
+        <v/>
+      </c>
+      <c r="K13" s="8">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I5, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="13">
+        <f>INDEX('📋 Детальный реестр'!B21:B26, 1)</f>
+        <v/>
+      </c>
+      <c r="D14" s="14">
+        <f>INDEX('📋 Детальный реестр'!C21:C26, 1)</f>
+        <v/>
+      </c>
+      <c r="E14" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F21:F26, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F21:F26, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>SUM('📋 Детальный реестр'!H21:H26)</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>SUM('📋 Детальный реестр'!G21:G26)</f>
+        <v/>
+      </c>
+      <c r="I14" s="15">
+        <f>SUM('📋 Детальный реестр'!I21:I26)</f>
+        <v/>
+      </c>
+      <c r="J14" s="15">
+        <f>SUM('📋 Детальный реестр'!M21:M26)</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I6, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="9">
+        <f>INDEX('📋 Детальный реестр'!B27:B32, 1)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>INDEX('📋 Детальный реестр'!C27:C32, 1)</f>
+        <v/>
+      </c>
+      <c r="E15" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F27:F32, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F15" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F27:F32, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G15" s="8">
+        <f>SUM('📋 Детальный реестр'!H27:H32)</f>
+        <v/>
+      </c>
+      <c r="H15" s="8">
+        <f>SUM('📋 Детальный реестр'!G27:G32)</f>
+        <v/>
+      </c>
+      <c r="I15" s="11">
+        <f>SUM('📋 Детальный реестр'!I27:I32)</f>
+        <v/>
+      </c>
+      <c r="J15" s="11">
+        <f>SUM('📋 Детальный реестр'!M27:M32)</f>
+        <v/>
+      </c>
+      <c r="K15" s="8">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I7, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="13">
+        <f>INDEX('📋 Детальный реестр'!B33:B38, 1)</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>INDEX('📋 Детальный реестр'!C33:C38, 1)</f>
+        <v/>
+      </c>
+      <c r="E16" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F33:F38, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F16" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F33:F38, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>SUM('📋 Детальный реестр'!H33:H38)</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>SUM('📋 Детальный реестр'!G33:G38)</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>SUM('📋 Детальный реестр'!I33:I38)</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>SUM('📋 Детальный реестр'!M33:M38)</f>
+        <v/>
+      </c>
+      <c r="K16" s="12">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I8, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>5243</v>
-      </c>
-      <c r="H11" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>8403</v>
-      </c>
-      <c r="J11" s="68" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L11" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="M11" s="41" t="inlineStr">
-        <is>
-          <t>🟢 0 фолл.</t>
-        </is>
-      </c>
-      <c r="N11" s="39">
-        <f>SUM(F11,H11,J11,K11,L11)</f>
-        <v/>
-      </c>
-      <c r="O11" s="42">
-        <f>G11+I11</f>
-        <v/>
-      </c>
-      <c r="P11" s="42" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q11" s="26" t="inlineStr">
-        <is>
-          <t>YouTube: 5,000 views</t>
-        </is>
-      </c>
-      <c r="R11" s="58" t="n"/>
-      <c r="S11" s="58" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="58" t="n"/>
-      <c r="B12" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" s="43" t="inlineStr">
-        <is>
-          <t>Ян Верса</t>
-        </is>
-      </c>
-      <c r="D12" s="34" t="inlineStr">
-        <is>
-          <t>Беларусь</t>
-        </is>
-      </c>
-      <c r="E12" s="44" t="inlineStr">
-        <is>
-          <t>Лёша</t>
-        </is>
-      </c>
-      <c r="F12" s="45" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>3570</v>
-      </c>
-      <c r="H12" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="I12" s="15" t="n">
-        <v>4200</v>
-      </c>
-      <c r="J12" s="68" t="n">
-        <v>5</v>
-      </c>
-      <c r="K12" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="M12" s="41" t="inlineStr">
-        <is>
-          <t>🟢 0 фолл.</t>
-        </is>
-      </c>
-      <c r="N12" s="45">
-        <f>SUM(F12,H12,J12,K12,L12)</f>
-        <v/>
-      </c>
-      <c r="O12" s="46">
-        <f>G12+I12</f>
-        <v/>
-      </c>
-      <c r="P12" s="46" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q12" s="29" t="inlineStr">
-        <is>
-          <t>YouTube: 1,100 views</t>
-        </is>
-      </c>
-      <c r="R12" s="58" t="n"/>
-      <c r="S12" s="58" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="58" t="n"/>
-      <c r="B13" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>Baraka Otieno</t>
-        </is>
-      </c>
-      <c r="D13" s="32" t="inlineStr">
-        <is>
-          <t>Кения</t>
-        </is>
-      </c>
-      <c r="E13" s="38" t="inlineStr">
-        <is>
-          <t>Саша</t>
-        </is>
-      </c>
-      <c r="F13" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>2717</v>
-      </c>
-      <c r="H13" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="47" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="L13" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="48" t="inlineStr">
+      <c r="C17" s="9">
+        <f>INDEX('📋 Детальный реестр'!B39:B44, 1)</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>INDEX('📋 Детальный реестр'!C39:C44, 1)</f>
+        <v/>
+      </c>
+      <c r="E17" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F39:F44, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F17" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F39:F44, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G17" s="8">
+        <f>SUM('📋 Детальный реестр'!H39:H44)</f>
+        <v/>
+      </c>
+      <c r="H17" s="8">
+        <f>SUM('📋 Детальный реестр'!G39:G44)</f>
+        <v/>
+      </c>
+      <c r="I17" s="11">
+        <f>SUM('📋 Детальный реестр'!I39:I44)</f>
+        <v/>
+      </c>
+      <c r="J17" s="11">
+        <f>SUM('📋 Детальный реестр'!M39:M44)</f>
+        <v/>
+      </c>
+      <c r="K17" s="8">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I9, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" s="13">
+        <f>INDEX('📋 Детальный реестр'!B45:B50, 1)</f>
+        <v/>
+      </c>
+      <c r="D18" s="14">
+        <f>INDEX('📋 Детальный реестр'!C45:C50, 1)</f>
+        <v/>
+      </c>
+      <c r="E18" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F45:F50, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F18" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F45:F50, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G18" s="12">
+        <f>SUM('📋 Детальный реестр'!H45:H50)</f>
+        <v/>
+      </c>
+      <c r="H18" s="12">
+        <f>SUM('📋 Детальный реестр'!G45:G50)</f>
+        <v/>
+      </c>
+      <c r="I18" s="15">
+        <f>SUM('📋 Детальный реестр'!I45:I50)</f>
+        <v/>
+      </c>
+      <c r="J18" s="15">
+        <f>SUM('📋 Детальный реестр'!M45:M50)</f>
+        <v/>
+      </c>
+      <c r="K18" s="12">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I10, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C19" s="9">
+        <f>INDEX('📋 Детальный реестр'!B51:B56, 1)</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>INDEX('📋 Детальный реестр'!C51:C56, 1)</f>
+        <v/>
+      </c>
+      <c r="E19" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F51:F56, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F19" s="8">
+        <f>COUNTIF('📋 Детальный реестр'!F51:F56, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G19" s="8">
+        <f>SUM('📋 Детальный реестр'!H51:H56)</f>
+        <v/>
+      </c>
+      <c r="H19" s="8">
+        <f>SUM('📋 Детальный реестр'!G51:G56)</f>
+        <v/>
+      </c>
+      <c r="I19" s="11">
+        <f>SUM('📋 Детальный реестр'!I51:I56)</f>
+        <v/>
+      </c>
+      <c r="J19" s="11">
+        <f>SUM('📋 Детальный реестр'!M51:M56)</f>
+        <v/>
+      </c>
+      <c r="K19" s="8">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I11, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="13">
+        <f>INDEX('📋 Детальный реестр'!B57:B62, 1)</f>
+        <v/>
+      </c>
+      <c r="D20" s="14">
+        <f>INDEX('📋 Детальный реестр'!C57:C62, 1)</f>
+        <v/>
+      </c>
+      <c r="E20" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F57:F62, "Активен")</f>
+        <v/>
+      </c>
+      <c r="F20" s="12">
+        <f>COUNTIF('📋 Детальный реестр'!F57:F62, "БАН")</f>
+        <v/>
+      </c>
+      <c r="G20" s="12">
+        <f>SUM('📋 Детальный реестр'!H57:H62)</f>
+        <v/>
+      </c>
+      <c r="H20" s="12">
+        <f>SUM('📋 Детальный реестр'!G57:G62)</f>
+        <v/>
+      </c>
+      <c r="I20" s="15">
+        <f>SUM('📋 Детальный реестр'!I57:I62)</f>
+        <v/>
+      </c>
+      <c r="J20" s="15">
+        <f>SUM('📋 Детальный реестр'!M57:M62)</f>
+        <v/>
+      </c>
+      <c r="K20" s="12">
+        <f>INDEX('🔍 Аудит и сверка спецов'!I12, 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="16" t="inlineStr"/>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N13" s="39">
-        <f>SUM(F13,H13,J13,K13,L13)</f>
-        <v/>
-      </c>
-      <c r="O13" s="42">
-        <f>G13+I13</f>
-        <v/>
-      </c>
-      <c r="P13" s="42" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q13" s="26" t="inlineStr">
-        <is>
-          <t>TikTok: 875 views</t>
-        </is>
-      </c>
-      <c r="R13" s="58" t="n"/>
-      <c r="S13" s="58" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="58" t="n"/>
-      <c r="B14" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>Grace Muthioni</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="inlineStr">
-        <is>
-          <t>Кения</t>
-        </is>
-      </c>
-      <c r="E14" s="44" t="inlineStr">
-        <is>
-          <t>Саша</t>
-        </is>
-      </c>
-      <c r="F14" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>1465</v>
-      </c>
-      <c r="H14" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="J14" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="48" t="inlineStr">
+      <c r="E21" s="19">
+        <f>SUM(E11:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>SUM(F11:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>SUM(G11:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="19">
+        <f>SUM(H11:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="20">
+        <f>SUM(I11:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="20">
+        <f>SUM(J11:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N14" s="45">
-        <f>SUM(F14,H14,J14,K14,L14)</f>
-        <v/>
-      </c>
-      <c r="O14" s="46">
-        <f>G14+I14</f>
-        <v/>
-      </c>
-      <c r="P14" s="46" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q14" s="29" t="inlineStr">
-        <is>
-          <t>TikTok: 528 views</t>
-        </is>
-      </c>
-      <c r="R14" s="58" t="n"/>
-      <c r="S14" s="58" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="58" t="n"/>
-      <c r="B15" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>Kaan Turan</t>
-        </is>
-      </c>
-      <c r="D15" s="32" t="inlineStr">
-        <is>
-          <t>Турция</t>
-        </is>
-      </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>Саша</t>
-        </is>
-      </c>
-      <c r="F15" s="39" t="n">
-        <v>8</v>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>5023</v>
-      </c>
-      <c r="H15" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>272</v>
-      </c>
-      <c r="J15" s="49" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="K15" s="47" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="L15" s="47" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="M15" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N15" s="39">
-        <f>SUM(F15,H15,J15,K15,L15)</f>
-        <v/>
-      </c>
-      <c r="O15" s="42">
-        <f>G15+I15</f>
-        <v/>
-      </c>
-      <c r="P15" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="26" t="inlineStr">
-        <is>
-          <t>TikTok: 1,089 views</t>
-        </is>
-      </c>
-      <c r="R15" s="58" t="n"/>
-      <c r="S15" s="58" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="58" t="n"/>
-      <c r="B16" s="34" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Melissa Kara</t>
-        </is>
-      </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>Турция</t>
-        </is>
-      </c>
-      <c r="E16" s="44" t="inlineStr">
-        <is>
-          <t>Саша</t>
-        </is>
-      </c>
-      <c r="F16" s="45" t="n">
-        <v>8</v>
-      </c>
-      <c r="G16" s="15" t="n">
-        <v>4351</v>
-      </c>
-      <c r="H16" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="15" t="n">
-        <v>1100</v>
-      </c>
-      <c r="J16" s="49" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="K16" s="47" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="L16" s="47" t="inlineStr">
-        <is>
-          <t>🔴 БАН</t>
-        </is>
-      </c>
-      <c r="M16" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N16" s="45">
-        <f>SUM(F16,H16,J16,K16,L16)</f>
-        <v/>
-      </c>
-      <c r="O16" s="46">
-        <f>G16+I16</f>
-        <v/>
-      </c>
-      <c r="P16" s="46" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q16" s="29" t="inlineStr">
-        <is>
-          <t>YouTube: 1,100 views</t>
-        </is>
-      </c>
-      <c r="R16" s="58" t="n"/>
-      <c r="S16" s="58" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="58" t="n"/>
-      <c r="B17" s="32" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>Асель Исакова</t>
-        </is>
-      </c>
-      <c r="D17" s="32" t="inlineStr">
-        <is>
-          <t>Кыргызстан</t>
-        </is>
-      </c>
-      <c r="E17" s="38" t="inlineStr">
-        <is>
-          <t>Сёма</t>
-        </is>
-      </c>
-      <c r="F17" s="39" t="n">
-        <v>7</v>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>23797</v>
-      </c>
-      <c r="H17" s="39" t="n">
-        <v>7</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>456323</v>
-      </c>
-      <c r="J17" s="68" t="n">
-        <v>4</v>
-      </c>
-      <c r="K17" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L17" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="M17" s="41" t="inlineStr">
-        <is>
-          <t>🟢 0 фолл.</t>
-        </is>
-      </c>
-      <c r="N17" s="39">
-        <f>SUM(F17,H17,J17,K17,L17)</f>
-        <v/>
-      </c>
-      <c r="O17" s="42">
-        <f>G17+I17</f>
-        <v/>
-      </c>
-      <c r="P17" s="42" t="n">
-        <v>596</v>
-      </c>
-      <c r="Q17" s="26" t="inlineStr">
-        <is>
-          <t>YouTube: 440,000 views</t>
-        </is>
-      </c>
-      <c r="R17" s="58" t="n"/>
-      <c r="S17" s="58" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="58" t="n"/>
-      <c r="B18" s="34" t="n">
-        <v>8</v>
-      </c>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>Тилек Асанов</t>
-        </is>
-      </c>
-      <c r="D18" s="34" t="inlineStr">
-        <is>
-          <t>Кыргызстан</t>
-        </is>
-      </c>
-      <c r="E18" s="44" t="inlineStr">
-        <is>
-          <t>Сёма</t>
-        </is>
-      </c>
-      <c r="F18" s="45" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>2241</v>
-      </c>
-      <c r="H18" s="45" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" s="15" t="n">
-        <v>8309</v>
-      </c>
-      <c r="J18" s="68" t="n">
-        <v>5</v>
-      </c>
-      <c r="K18" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L18" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="M18" s="41" t="inlineStr">
-        <is>
-          <t>🟢 0 фолл.</t>
-        </is>
-      </c>
-      <c r="N18" s="45">
-        <f>SUM(F18,H18,J18,K18,L18)</f>
-        <v/>
-      </c>
-      <c r="O18" s="46">
-        <f>G18+I18</f>
-        <v/>
-      </c>
-      <c r="P18" s="46" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q18" s="29" t="inlineStr">
-        <is>
-          <t>YouTube: 3,200 views</t>
-        </is>
-      </c>
-      <c r="R18" s="58" t="n"/>
-      <c r="S18" s="58" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="58" t="n"/>
-      <c r="B19" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
-        <is>
-          <t>Lori Bennet</t>
-        </is>
-      </c>
-      <c r="D19" s="32" t="inlineStr">
-        <is>
-          <t>Америка</t>
-        </is>
-      </c>
-      <c r="E19" s="38" t="inlineStr">
-        <is>
-          <t>Даник</t>
-        </is>
-      </c>
-      <c r="F19" s="39" t="n">
-        <v>6</v>
-      </c>
-      <c r="G19" s="11" t="n">
-        <v>1217</v>
-      </c>
-      <c r="H19" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>2721</v>
-      </c>
-      <c r="J19" s="68" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="41" t="inlineStr">
-        <is>
-          <t>🟢 2 фолл.</t>
-        </is>
-      </c>
-      <c r="N19" s="39">
-        <f>SUM(F19,H19,J19,K19,L19)</f>
-        <v/>
-      </c>
-      <c r="O19" s="42">
-        <f>G19+I19</f>
-        <v/>
-      </c>
-      <c r="P19" s="42" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q19" s="26" t="inlineStr">
-        <is>
-          <t>YouTube: 1,400 views</t>
-        </is>
-      </c>
-      <c r="R19" s="58" t="n"/>
-      <c r="S19" s="58" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="58" t="n"/>
-      <c r="B20" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="C20" s="43" t="inlineStr">
-        <is>
-          <t>Vida</t>
-        </is>
-      </c>
-      <c r="D20" s="34" t="inlineStr">
-        <is>
-          <t>Америка</t>
-        </is>
-      </c>
-      <c r="E20" s="44" t="inlineStr">
-        <is>
-          <t>Артур</t>
-        </is>
-      </c>
-      <c r="F20" s="45" t="n">
-        <v>56</v>
-      </c>
-      <c r="G20" s="15" t="n">
-        <v>28464</v>
-      </c>
-      <c r="H20" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K20" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L20" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M20" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N20" s="45">
-        <f>SUM(F20,H20,J20,K20,L20)</f>
-        <v/>
-      </c>
-      <c r="O20" s="46">
-        <f>G20+I20</f>
-        <v/>
-      </c>
-      <c r="P20" s="46" t="n">
-        <v>2936</v>
-      </c>
-      <c r="Q20" s="29" t="inlineStr">
-        <is>
-          <t>TikTok: 985 views</t>
-        </is>
-      </c>
-      <c r="R20" s="58" t="n"/>
-      <c r="S20" s="58" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="58" t="n"/>
-      <c r="B21" s="16" t="inlineStr"/>
-      <c r="C21" s="73" t="inlineStr">
-        <is>
-          <t>ИТОГО ПО СЕТКЕ</t>
-        </is>
-      </c>
-      <c r="D21" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="75" t="inlineStr">
-        <is>
-          <t>5 спецов</t>
-        </is>
-      </c>
-      <c r="F21" s="76">
-        <f>SUM(F11:F20)</f>
-        <v/>
-      </c>
-      <c r="G21" s="77">
-        <f>SUM(G11:G20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="76">
-        <f>SUM(H11:H20)</f>
-        <v/>
-      </c>
-      <c r="I21" s="77">
-        <f>SUM(I11:I20)</f>
-        <v/>
-      </c>
-      <c r="J21" s="78" t="inlineStr">
-        <is>
-          <t>7 акт / 2 бан</t>
-        </is>
-      </c>
-      <c r="K21" s="74" t="inlineStr">
-        <is>
-          <t>7 акт / 3 бан</t>
-        </is>
-      </c>
-      <c r="L21" s="74" t="inlineStr">
-        <is>
-          <t>7 акт / 2 бан</t>
-        </is>
-      </c>
-      <c r="M21" s="74" t="inlineStr">
-        <is>
-          <t>5 акт / 0 бан</t>
-        </is>
-      </c>
-      <c r="N21" s="76">
-        <f>SUM(N11:N20)</f>
-        <v/>
-      </c>
-      <c r="O21" s="77">
-        <f>SUM(O11:O20)</f>
-        <v/>
-      </c>
-      <c r="P21" s="77">
-        <f>SUM(P11:P20)</f>
-        <v/>
-      </c>
-      <c r="Q21" s="79" t="inlineStr">
-        <is>
-          <t>Асель Исакова (3.8k)</t>
-        </is>
-      </c>
-      <c r="R21" s="58" t="n"/>
-      <c r="S21" s="58" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="58" t="n"/>
-      <c r="B22" s="58" t="n"/>
-      <c r="C22" s="58" t="n"/>
-      <c r="D22" s="58" t="n"/>
-      <c r="E22" s="58" t="n"/>
-      <c r="F22" s="58" t="n"/>
-      <c r="G22" s="58" t="n"/>
-      <c r="H22" s="58" t="n"/>
-      <c r="I22" s="58" t="n"/>
-      <c r="J22" s="58" t="n"/>
-      <c r="K22" s="58" t="n"/>
-      <c r="L22" s="58" t="n"/>
-      <c r="M22" s="58" t="n"/>
-      <c r="N22" s="58" t="n"/>
-      <c r="O22" s="58" t="n"/>
-      <c r="P22" s="58" t="n"/>
-      <c r="Q22" s="58" t="n"/>
-      <c r="R22" s="58" t="n"/>
-      <c r="S22" s="58" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="58" t="n"/>
-      <c r="B23" s="58" t="n"/>
-      <c r="C23" s="58" t="n"/>
-      <c r="D23" s="58" t="n"/>
-      <c r="E23" s="58" t="n"/>
-      <c r="F23" s="58" t="n"/>
-      <c r="G23" s="58" t="n"/>
-      <c r="H23" s="58" t="n"/>
-      <c r="I23" s="58" t="n"/>
-      <c r="J23" s="58" t="n"/>
-      <c r="K23" s="58" t="n"/>
-      <c r="L23" s="58" t="n"/>
-      <c r="M23" s="58" t="n"/>
-      <c r="N23" s="58" t="n"/>
-      <c r="O23" s="58" t="n"/>
-      <c r="P23" s="58" t="n"/>
-      <c r="Q23" s="58" t="n"/>
-      <c r="R23" s="58" t="n"/>
-      <c r="S23" s="58" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="58" t="n"/>
-      <c r="B24" s="58" t="n"/>
-      <c r="C24" s="58" t="n"/>
-      <c r="D24" s="58" t="n"/>
-      <c r="E24" s="58" t="n"/>
-      <c r="F24" s="58" t="n"/>
-      <c r="G24" s="58" t="n"/>
-      <c r="H24" s="58" t="n"/>
-      <c r="I24" s="58" t="n"/>
-      <c r="J24" s="58" t="n"/>
-      <c r="K24" s="58" t="n"/>
-      <c r="L24" s="58" t="n"/>
-      <c r="M24" s="58" t="n"/>
-      <c r="N24" s="58" t="n"/>
-      <c r="O24" s="58" t="n"/>
-      <c r="P24" s="58" t="n"/>
-      <c r="Q24" s="58" t="n"/>
-      <c r="R24" s="58" t="n"/>
-      <c r="S24" s="58" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="58" t="n"/>
-      <c r="B25" s="58" t="n"/>
-      <c r="C25" s="58" t="n"/>
-      <c r="D25" s="58" t="n"/>
-      <c r="E25" s="58" t="n"/>
-      <c r="F25" s="58" t="n"/>
-      <c r="G25" s="58" t="n"/>
-      <c r="H25" s="58" t="n"/>
-      <c r="I25" s="58" t="n"/>
-      <c r="J25" s="58" t="n"/>
-      <c r="K25" s="58" t="n"/>
-      <c r="L25" s="58" t="n"/>
-      <c r="M25" s="58" t="n"/>
-      <c r="N25" s="58" t="n"/>
-      <c r="O25" s="58" t="n"/>
-      <c r="P25" s="58" t="n"/>
-      <c r="Q25" s="58" t="n"/>
-      <c r="R25" s="58" t="n"/>
-      <c r="S25" s="58" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="58" t="n"/>
-      <c r="B26" s="58" t="n"/>
-      <c r="C26" s="58" t="n"/>
-      <c r="D26" s="58" t="n"/>
-      <c r="E26" s="58" t="n"/>
-      <c r="F26" s="58" t="n"/>
-      <c r="G26" s="58" t="n"/>
-      <c r="H26" s="58" t="n"/>
-      <c r="I26" s="58" t="n"/>
-      <c r="J26" s="58" t="n"/>
-      <c r="K26" s="58" t="n"/>
-      <c r="L26" s="58" t="n"/>
-      <c r="M26" s="58" t="n"/>
-      <c r="N26" s="58" t="n"/>
-      <c r="O26" s="58" t="n"/>
-      <c r="P26" s="58" t="n"/>
-      <c r="Q26" s="58" t="n"/>
-      <c r="R26" s="58" t="n"/>
-      <c r="S26" s="58" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="58" t="n"/>
-      <c r="B27" s="58" t="n"/>
-      <c r="C27" s="58" t="n"/>
-      <c r="D27" s="58" t="n"/>
-      <c r="E27" s="58" t="n"/>
-      <c r="F27" s="58" t="n"/>
-      <c r="G27" s="58" t="n"/>
-      <c r="H27" s="58" t="n"/>
-      <c r="I27" s="58" t="n"/>
-      <c r="J27" s="58" t="n"/>
-      <c r="K27" s="58" t="n"/>
-      <c r="L27" s="58" t="n"/>
-      <c r="M27" s="58" t="n"/>
-      <c r="N27" s="58" t="n"/>
-      <c r="O27" s="58" t="n"/>
-      <c r="P27" s="58" t="n"/>
-      <c r="Q27" s="58" t="n"/>
-      <c r="R27" s="58" t="n"/>
-      <c r="S27" s="58" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="58" t="n"/>
-      <c r="B28" s="58" t="n"/>
-      <c r="C28" s="58" t="n"/>
-      <c r="D28" s="58" t="n"/>
-      <c r="E28" s="58" t="n"/>
-      <c r="F28" s="58" t="n"/>
-      <c r="G28" s="58" t="n"/>
-      <c r="H28" s="58" t="n"/>
-      <c r="I28" s="58" t="n"/>
-      <c r="J28" s="58" t="n"/>
-      <c r="K28" s="58" t="n"/>
-      <c r="L28" s="58" t="n"/>
-      <c r="M28" s="58" t="n"/>
-      <c r="N28" s="58" t="n"/>
-      <c r="O28" s="58" t="n"/>
-      <c r="P28" s="58" t="n"/>
-      <c r="Q28" s="58" t="n"/>
-      <c r="R28" s="58" t="n"/>
-      <c r="S28" s="58" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="58" t="n"/>
-      <c r="B29" s="58" t="n"/>
-      <c r="C29" s="58" t="n"/>
-      <c r="D29" s="58" t="n"/>
-      <c r="E29" s="58" t="n"/>
-      <c r="F29" s="58" t="n"/>
-      <c r="G29" s="58" t="n"/>
-      <c r="H29" s="58" t="n"/>
-      <c r="I29" s="58" t="n"/>
-      <c r="J29" s="58" t="n"/>
-      <c r="K29" s="58" t="n"/>
-      <c r="L29" s="58" t="n"/>
-      <c r="M29" s="58" t="n"/>
-      <c r="N29" s="58" t="n"/>
-      <c r="O29" s="58" t="n"/>
-      <c r="P29" s="58" t="n"/>
-      <c r="Q29" s="58" t="n"/>
-      <c r="R29" s="58" t="n"/>
-      <c r="S29" s="58" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2027,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R62"/>
+  <dimension ref="A2:R62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2050,13 +1304,6 @@
     <col width="25" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="81" t="inlineStr">
-        <is>
-          <t>📋 РЕЕСТР 60 АККАУНТОВ ИНФЛЮЕНСЕРОВ (Дата и время выгрузки: 07.09.2026 в 10:20:31 МСК)</t>
-        </is>
-      </c>
-    </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
@@ -2158,7 +1405,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C3" s="53" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2173,7 +1420,7 @@
           <t>https://www.tiktok.com/@yanveras13</t>
         </is>
       </c>
-      <c r="F3" s="41" t="inlineStr">
+      <c r="F3" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2185,7 +1432,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>5243</v>
+        <v>5268</v>
       </c>
       <c r="J3" s="11" t="n">
         <v>136</v>
@@ -2205,7 +1452,7 @@
         <v>0</v>
       </c>
       <c r="O3" s="11" t="n">
-        <v>488</v>
+        <v>552</v>
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
@@ -2230,7 +1477,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C4" s="53" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2245,7 +1492,7 @@
           <t>https://youtube.com/channel/UCn-t5Z16uoP60hkWQQ7d_Tg</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2298,7 +1545,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C5" s="53" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2313,7 +1560,7 @@
           <t>https://www.instagram.com/anveras509</t>
         </is>
       </c>
-      <c r="F5" s="41" t="inlineStr">
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2325,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="J5" s="11" t="n">
         <v>0</v>
@@ -2366,7 +1613,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C6" s="53" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2381,19 +1628,19 @@
           <t>https://www.facebook.com/share/1BMagQvaoE/</t>
         </is>
       </c>
-      <c r="F6" s="41" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G6" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>615</v>
+        <v>718</v>
       </c>
       <c r="J6" s="11" t="n">
         <v>43</v>
@@ -2434,7 +1681,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C7" s="53" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2446,16 +1693,16 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@alesabut</t>
-        </is>
-      </c>
-      <c r="F7" s="41" t="inlineStr">
+          <t>https://www.threads.net/@alesabut</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G7" s="32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7" s="32" t="n">
         <v>0</v>
@@ -2502,7 +1749,7 @@
           <t>Алеся Бут (Беларусь)</t>
         </is>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2517,7 +1764,7 @@
           <t>https://x.com/ft73v5</t>
         </is>
       </c>
-      <c r="F8" s="41" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2570,7 +1817,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C9" s="54" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2585,7 +1832,7 @@
           <t>https://www.tiktok.com/@alesyabyt</t>
         </is>
       </c>
-      <c r="F9" s="41" t="inlineStr">
+      <c r="F9" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2597,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>3570</v>
+        <v>3605</v>
       </c>
       <c r="J9" s="15" t="n">
         <v>550</v>
@@ -2617,7 +1864,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="15" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="P9" s="14" t="inlineStr">
         <is>
@@ -2642,7 +1889,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C10" s="54" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2657,7 +1904,7 @@
           <t>https://youtube.com/channel/UCxgk7mDrX45Wb9Wv61hO75w</t>
         </is>
       </c>
-      <c r="F10" s="41" t="inlineStr">
+      <c r="F10" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2710,7 +1957,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2725,7 +1972,7 @@
           <t>https://www.instagram.com/alesabut</t>
         </is>
       </c>
-      <c r="F11" s="41" t="inlineStr">
+      <c r="F11" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2778,7 +2025,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C12" s="54" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2793,19 +2040,19 @@
           <t>https://www.facebook.com/share/1GbKg4Tp5n/</t>
         </is>
       </c>
-      <c r="F12" s="41" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G12" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="15" t="n">
-        <v>0</v>
+        <v>248</v>
       </c>
       <c r="J12" s="15" t="n">
         <v>0</v>
@@ -2846,7 +2093,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C13" s="54" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2858,16 +2105,16 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@anveras509</t>
-        </is>
-      </c>
-      <c r="F13" s="41" t="inlineStr">
+          <t>https://www.threads.net/@anveras509</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G13" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H13" s="34" t="n">
         <v>0</v>
@@ -2887,7 +2134,7 @@
         </is>
       </c>
       <c r="M13" s="15" t="n">
-        <v>0</v>
+        <v>509</v>
       </c>
       <c r="N13" s="23" t="n">
         <v>0</v>
@@ -2914,7 +2161,7 @@
           <t>Ян Верса (Беларусь)</t>
         </is>
       </c>
-      <c r="C14" s="54" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Лёша</t>
         </is>
@@ -2929,7 +2176,7 @@
           <t>https://x.com/neaz8b</t>
         </is>
       </c>
-      <c r="F14" s="41" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -2982,7 +2229,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C15" s="53" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -2997,19 +2244,19 @@
           <t>https://www.tiktok.com/@baraka.otieno8</t>
         </is>
       </c>
-      <c r="F15" s="41" t="inlineStr">
+      <c r="F15" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G15" s="32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H15" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>2717</v>
+        <v>3229</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>47</v>
@@ -3029,7 +2276,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="11" t="n">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
@@ -3054,7 +2301,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C16" s="53" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3069,7 +2316,7 @@
           <t>https://www.youtube.com/@BarakaOtieno-t9y</t>
         </is>
       </c>
-      <c r="F16" s="41" t="inlineStr">
+      <c r="F16" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3122,7 +2369,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C17" s="53" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3137,7 +2384,7 @@
           <t>https://www.instagram.com/otienobarakaa</t>
         </is>
       </c>
-      <c r="F17" s="41" t="inlineStr">
+      <c r="F17" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3190,7 +2437,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C18" s="53" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3205,9 +2452,9 @@
           <t>https://www.facebook.com/profile.php?id=61594225224413</t>
         </is>
       </c>
-      <c r="F18" s="47" t="inlineStr">
-        <is>
-          <t>БАН</t>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>Активен</t>
         </is>
       </c>
       <c r="G18" s="32" t="n">
@@ -3258,7 +2505,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C19" s="53" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3270,10 +2517,10 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@otienobarakaa</t>
-        </is>
-      </c>
-      <c r="F19" s="41" t="inlineStr">
+          <t>https://www.threads.net/@otienobarakaa</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3326,7 +2573,7 @@
           <t>Baraka Otieno (Кения)</t>
         </is>
       </c>
-      <c r="C20" s="53" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3337,7 +2584,7 @@
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr"/>
-      <c r="F20" s="55" t="inlineStr">
+      <c r="F20" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -3390,7 +2637,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C21" s="54" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3405,19 +2652,19 @@
           <t>https://www.tiktok.com/@grace.muthioni</t>
         </is>
       </c>
-      <c r="F21" s="41" t="inlineStr">
+      <c r="F21" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G21" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H21" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>1465</v>
+        <v>1511</v>
       </c>
       <c r="J21" s="15" t="n">
         <v>52</v>
@@ -3437,7 +2684,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="15" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="P21" s="14" t="inlineStr">
         <is>
@@ -3462,7 +2709,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C22" s="54" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3477,7 +2724,7 @@
           <t>https://www.youtube.com/@GraceMuthioni</t>
         </is>
       </c>
-      <c r="F22" s="41" t="inlineStr">
+      <c r="F22" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3530,7 +2777,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C23" s="54" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3545,7 +2792,7 @@
           <t>https://www.instagram.com/gracemuthioni</t>
         </is>
       </c>
-      <c r="F23" s="41" t="inlineStr">
+      <c r="F23" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3598,7 +2845,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C24" s="54" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3613,13 +2860,13 @@
           <t>https://www.facebook.com/share/19Yipg1q9R/</t>
         </is>
       </c>
-      <c r="F24" s="41" t="inlineStr">
+      <c r="F24" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G24" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" s="34" t="n">
         <v>0</v>
@@ -3666,7 +2913,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C25" s="54" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3678,10 +2925,10 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@gracemuthioni</t>
-        </is>
-      </c>
-      <c r="F25" s="41" t="inlineStr">
+          <t>https://www.threads.net/@gracemuthioni</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3734,7 +2981,7 @@
           <t>Grace Muthioni (Кения)</t>
         </is>
       </c>
-      <c r="C26" s="54" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3745,7 +2992,7 @@
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr"/>
-      <c r="F26" s="55" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -3798,7 +3045,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C27" s="53" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3813,19 +3060,19 @@
           <t>https://www.tiktok.com/@kaan.turan225</t>
         </is>
       </c>
-      <c r="F27" s="41" t="inlineStr">
+      <c r="F27" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G27" s="32" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H27" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>5023</v>
+        <v>5326</v>
       </c>
       <c r="J27" s="11" t="n">
         <v>179</v>
@@ -3845,7 +3092,7 @@
         <v>0</v>
       </c>
       <c r="O27" s="11" t="n">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
@@ -3870,7 +3117,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C28" s="53" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3885,7 +3132,7 @@
           <t>https://www.youtube.com/@KAANTURAN-e5k</t>
         </is>
       </c>
-      <c r="F28" s="41" t="inlineStr">
+      <c r="F28" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -3897,7 +3144,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J28" s="11" t="n">
         <v>110</v>
@@ -3938,7 +3185,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C29" s="53" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -3953,7 +3200,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F29" s="47" t="inlineStr">
+      <c r="F29" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4006,7 +3253,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C30" s="53" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4021,7 +3268,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F30" s="47" t="inlineStr">
+      <c r="F30" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4074,7 +3321,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C31" s="53" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4089,7 +3336,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F31" s="47" t="inlineStr">
+      <c r="F31" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4142,7 +3389,7 @@
           <t>Kaan Turan (Турция)</t>
         </is>
       </c>
-      <c r="C32" s="53" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4153,7 +3400,7 @@
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr"/>
-      <c r="F32" s="55" t="inlineStr">
+      <c r="F32" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -4206,7 +3453,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C33" s="54" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4221,19 +3468,19 @@
           <t>https://www.tiktok.com/@melissa.kara47</t>
         </is>
       </c>
-      <c r="F33" s="41" t="inlineStr">
+      <c r="F33" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G33" s="34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H33" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>4351</v>
+        <v>4385</v>
       </c>
       <c r="J33" s="15" t="n">
         <v>44</v>
@@ -4253,7 +3500,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="15" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="P33" s="14" t="inlineStr">
         <is>
@@ -4278,7 +3525,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C34" s="54" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4293,7 +3540,7 @@
           <t>https://www.youtube.com/@MelissaKaraaa</t>
         </is>
       </c>
-      <c r="F34" s="41" t="inlineStr">
+      <c r="F34" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -4346,7 +3593,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C35" s="54" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4361,7 +3608,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F35" s="47" t="inlineStr">
+      <c r="F35" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4414,7 +3661,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C36" s="54" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4429,7 +3676,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F36" s="47" t="inlineStr">
+      <c r="F36" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4482,7 +3729,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C37" s="54" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4497,7 +3744,7 @@
           <t>Бан</t>
         </is>
       </c>
-      <c r="F37" s="47" t="inlineStr">
+      <c r="F37" s="36" t="inlineStr">
         <is>
           <t>БАН</t>
         </is>
@@ -4550,7 +3797,7 @@
           <t>Melissa Kara (Турция)</t>
         </is>
       </c>
-      <c r="C38" s="54" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Саша</t>
         </is>
@@ -4561,7 +3808,7 @@
         </is>
       </c>
       <c r="E38" s="14" t="inlineStr"/>
-      <c r="F38" s="55" t="inlineStr">
+      <c r="F38" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -4614,7 +3861,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C39" s="53" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4626,22 +3873,22 @@
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>tiktok.com/@asel.isakova.077</t>
-        </is>
-      </c>
-      <c r="F39" s="41" t="inlineStr">
+          <t>https://www.tiktok.com/@asel.isakova.077</t>
+        </is>
+      </c>
+      <c r="F39" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G39" s="32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H39" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>23797</v>
+        <v>32539</v>
       </c>
       <c r="J39" s="11" t="n">
         <v>56</v>
@@ -4655,13 +3902,13 @@
         </is>
       </c>
       <c r="M39" s="11" t="n">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="N39" s="22" t="n">
         <v>0</v>
       </c>
       <c r="O39" s="11" t="n">
-        <v>1302</v>
+        <v>1989</v>
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
@@ -4682,7 +3929,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C40" s="53" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4697,19 +3944,19 @@
           <t>https://www.youtube.com/@%D0%90%D1%81%D0%B5%D0%BB%D1%8C%D0%98%D1%81%D0%B0%D0%BA%D0%BE%D0%B2%D0%B0-%D1%824%D1%86</t>
         </is>
       </c>
-      <c r="F40" s="41" t="inlineStr">
+      <c r="F40" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G40" s="32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H40" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>456323</v>
+        <v>720296</v>
       </c>
       <c r="J40" s="11" t="n">
         <v>9</v>
@@ -4723,7 +3970,7 @@
         </is>
       </c>
       <c r="M40" s="11" t="n">
-        <v>519</v>
+        <v>782</v>
       </c>
       <c r="N40" s="22" t="n">
         <v>0</v>
@@ -4746,7 +3993,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C41" s="53" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4761,13 +4008,13 @@
           <t>https://www.instagram.com/aseli_sakova?igsi=MTFvN2w4cHl2enQ2bg==</t>
         </is>
       </c>
-      <c r="F41" s="41" t="inlineStr">
+      <c r="F41" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G41" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H41" s="32" t="n">
         <v>0</v>
@@ -4810,7 +4057,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C42" s="53" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4825,19 +4072,19 @@
           <t>https://www.facebook.com/share/19YrNEtvbj/</t>
         </is>
       </c>
-      <c r="F42" s="41" t="inlineStr">
+      <c r="F42" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G42" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H42" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>1938</v>
+        <v>3446</v>
       </c>
       <c r="J42" s="11" t="n">
         <v>214</v>
@@ -4874,7 +4121,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C43" s="53" t="inlineStr">
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4886,10 +4133,10 @@
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@aseli_sakova</t>
-        </is>
-      </c>
-      <c r="F43" s="41" t="inlineStr">
+          <t>https://www.threads.net/@aseli_sakova</t>
+        </is>
+      </c>
+      <c r="F43" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -4915,7 +4162,7 @@
         </is>
       </c>
       <c r="M43" s="11" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="N43" s="22" t="n">
         <v>0</v>
@@ -4938,7 +4185,7 @@
           <t>Асель Исакова (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C44" s="53" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -4953,7 +4200,7 @@
           <t>https://x.com/mxhp8u</t>
         </is>
       </c>
-      <c r="F44" s="41" t="inlineStr">
+      <c r="F44" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5002,7 +4249,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C45" s="54" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5014,10 +4261,10 @@
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>tiktok.com/@tilek.asanov.77</t>
-        </is>
-      </c>
-      <c r="F45" s="41" t="inlineStr">
+          <t>https://www.tiktok.com/@tilek.asanov.77</t>
+        </is>
+      </c>
+      <c r="F45" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5029,7 +4276,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>2241</v>
+        <v>2287</v>
       </c>
       <c r="J45" s="15" t="n">
         <v>24</v>
@@ -5049,7 +4296,7 @@
         <v>0</v>
       </c>
       <c r="O45" s="15" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="P45" s="14" t="inlineStr">
         <is>
@@ -5070,7 +4317,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C46" s="54" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5085,7 +4332,7 @@
           <t>https://www.youtube.com/@tilek.asanov</t>
         </is>
       </c>
-      <c r="F46" s="41" t="inlineStr">
+      <c r="F46" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5097,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="15" t="n">
-        <v>8309</v>
+        <v>8411</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>271</v>
@@ -5134,7 +4381,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C47" s="54" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5149,13 +4396,13 @@
           <t>https://www.instagram.com/tile.kasanov?igsi=MThrajZrcWI3OW5qaA==</t>
         </is>
       </c>
-      <c r="F47" s="41" t="inlineStr">
+      <c r="F47" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G47" s="34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H47" s="34" t="n">
         <v>0</v>
@@ -5198,7 +4445,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C48" s="54" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5213,19 +4460,19 @@
           <t>https://www.facebook.com/share/1GmysHvXZ5/</t>
         </is>
       </c>
-      <c r="F48" s="41" t="inlineStr">
+      <c r="F48" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G48" s="34" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H48" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="15" t="n">
-        <v>787</v>
+        <v>1624</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>84</v>
@@ -5262,7 +4509,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C49" s="54" t="inlineStr">
+      <c r="C49" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5274,10 +4521,10 @@
       </c>
       <c r="E49" s="14" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@tile.kasanov</t>
-        </is>
-      </c>
-      <c r="F49" s="41" t="inlineStr">
+          <t>https://www.threads.net/@tile.kasanov</t>
+        </is>
+      </c>
+      <c r="F49" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5326,7 +4573,7 @@
           <t>Тилек Асанов (Кыргызстан)</t>
         </is>
       </c>
-      <c r="C50" s="54" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>Сёма</t>
         </is>
@@ -5341,7 +4588,7 @@
           <t>https://x.com/7jfe13</t>
         </is>
       </c>
-      <c r="F50" s="41" t="inlineStr">
+      <c r="F50" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5390,7 +4637,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C51" s="53" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5405,7 +4652,7 @@
           <t>https://www.tiktok.com/@lori.bennett08</t>
         </is>
       </c>
-      <c r="F51" s="41" t="inlineStr">
+      <c r="F51" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5417,7 +4664,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>1217</v>
+        <v>1309</v>
       </c>
       <c r="J51" s="11" t="n">
         <v>320</v>
@@ -5437,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="O51" s="11" t="n">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="P51" s="10" t="inlineStr">
         <is>
@@ -5458,7 +4705,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C52" s="53" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5473,7 +4720,7 @@
           <t>https://www.youtube.com/@LoriBennett-r5m</t>
         </is>
       </c>
-      <c r="F52" s="41" t="inlineStr">
+      <c r="F52" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5485,7 +4732,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>2721</v>
+        <v>2720</v>
       </c>
       <c r="J52" s="11" t="n">
         <v>15</v>
@@ -5522,7 +4769,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C53" s="53" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5537,7 +4784,7 @@
           <t>https://www.instagram.com/Lori_bennett14</t>
         </is>
       </c>
-      <c r="F53" s="41" t="inlineStr">
+      <c r="F53" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5549,7 +4796,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="J53" s="11" t="n">
         <v>0</v>
@@ -5586,7 +4833,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C54" s="53" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5601,13 +4848,13 @@
           <t>https://www.facebook.com/people/Lori-Bennett/</t>
         </is>
       </c>
-      <c r="F54" s="41" t="inlineStr">
+      <c r="F54" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G54" s="32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H54" s="32" t="n">
         <v>0</v>
@@ -5650,7 +4897,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C55" s="53" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5662,16 +4909,16 @@
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>https://www.threads.com/@lori_bennett14</t>
-        </is>
-      </c>
-      <c r="F55" s="41" t="inlineStr">
+          <t>https://www.threads.net/@lori_bennett14</t>
+        </is>
+      </c>
+      <c r="F55" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G55" s="32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H55" s="32" t="n">
         <v>0</v>
@@ -5691,7 +4938,7 @@
         </is>
       </c>
       <c r="M55" s="11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="N55" s="22" t="n">
         <v>0</v>
@@ -5714,7 +4961,7 @@
           <t>Lori Bennet (Америка)</t>
         </is>
       </c>
-      <c r="C56" s="53" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
         <is>
           <t>Даник</t>
         </is>
@@ -5729,7 +4976,7 @@
           <t>https://x.com/LoriBennet7jcr</t>
         </is>
       </c>
-      <c r="F56" s="41" t="inlineStr">
+      <c r="F56" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
@@ -5755,7 +5002,7 @@
         </is>
       </c>
       <c r="M56" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N56" s="22" t="n">
         <v>0</v>
@@ -5778,7 +5025,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C57" s="54" t="inlineStr">
+      <c r="C57" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -5793,19 +5040,19 @@
           <t>https://www.tiktok.com/@vida_morales?_r=1&amp;_t=ZS-99RwjrUI14c</t>
         </is>
       </c>
-      <c r="F57" s="41" t="inlineStr">
+      <c r="F57" s="33" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
       <c r="G57" s="34" t="n">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="H57" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I57" s="15" t="n">
-        <v>4914</v>
+        <v>28526</v>
       </c>
       <c r="J57" s="15" t="n">
         <v>965</v>
@@ -5819,13 +5066,13 @@
         </is>
       </c>
       <c r="M57" s="15" t="n">
-        <v>2935</v>
+        <v>2936</v>
       </c>
       <c r="N57" s="23" t="n">
         <v>0</v>
       </c>
       <c r="O57" s="15" t="n">
-        <v>31100</v>
+        <v>31200</v>
       </c>
       <c r="P57" s="14" t="inlineStr">
         <is>
@@ -5846,7 +5093,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C58" s="54" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -5857,7 +5104,7 @@
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr"/>
-      <c r="F58" s="55" t="inlineStr">
+      <c r="F58" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -5906,7 +5153,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C59" s="54" t="inlineStr">
+      <c r="C59" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -5917,7 +5164,7 @@
         </is>
       </c>
       <c r="E59" s="14" t="inlineStr"/>
-      <c r="F59" s="55" t="inlineStr">
+      <c r="F59" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -5966,7 +5213,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C60" s="54" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -5977,7 +5224,7 @@
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr"/>
-      <c r="F60" s="55" t="inlineStr">
+      <c r="F60" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -6026,7 +5273,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C61" s="54" t="inlineStr">
+      <c r="C61" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -6037,7 +5284,7 @@
         </is>
       </c>
       <c r="E61" s="14" t="inlineStr"/>
-      <c r="F61" s="55" t="inlineStr">
+      <c r="F61" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -6086,7 +5333,7 @@
           <t>Vida (Америка)</t>
         </is>
       </c>
-      <c r="C62" s="54" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
         <is>
           <t>Артур</t>
         </is>
@@ -6097,7 +5344,7 @@
         </is>
       </c>
       <c r="E62" s="14" t="inlineStr"/>
-      <c r="F62" s="55" t="inlineStr">
+      <c r="F62" s="35" t="inlineStr">
         <is>
           <t>Нет ссылки</t>
         </is>
@@ -6164,9 +5411,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="82" t="inlineStr">
-        <is>
-          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ VS ФАКТЫ (Сформировано: 07.09.2026 в 10:20:31 МСК)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>МОДУЛЬ СВЕРКИ И АНТИФРОДА: ЗАЯВЛЕНИЯ СПЕЦИАЛИСТОВ VS РЕАЛЬНЫЕ ФАКТЫ</t>
         </is>
       </c>
     </row>
@@ -6223,14 +5470,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="56" t="n">
+      <c r="A3" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="53">
+      <c r="B3" s="26">
         <f>INDEX('📋 Детальный реестр'!C3:C8, 1)</f>
         <v/>
       </c>
-      <c r="C3" s="37">
+      <c r="C3" s="9">
         <f>INDEX('📋 Детальный реестр'!B3:B8, 1)</f>
         <v/>
       </c>
@@ -6259,14 +5506,14 @@
       <c r="J3" s="26" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="57" t="n">
+      <c r="A4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="54">
+      <c r="B4" s="29">
         <f>INDEX('📋 Детальный реестр'!C9:C14, 1)</f>
         <v/>
       </c>
-      <c r="C4" s="43">
+      <c r="C4" s="13">
         <f>INDEX('📋 Детальный реестр'!B9:B14, 1)</f>
         <v/>
       </c>
@@ -6295,14 +5542,14 @@
       <c r="J4" s="29" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="56" t="n">
+      <c r="A5" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="53">
+      <c r="B5" s="26">
         <f>INDEX('📋 Детальный реестр'!C15:C20, 1)</f>
         <v/>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="9">
         <f>INDEX('📋 Детальный реестр'!B15:B20, 1)</f>
         <v/>
       </c>
@@ -6331,14 +5578,14 @@
       <c r="J5" s="26" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="57" t="n">
+      <c r="A6" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="54">
+      <c r="B6" s="29">
         <f>INDEX('📋 Детальный реестр'!C21:C26, 1)</f>
         <v/>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="13">
         <f>INDEX('📋 Детальный реестр'!B21:B26, 1)</f>
         <v/>
       </c>
@@ -6367,14 +5614,14 @@
       <c r="J6" s="29" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="56" t="n">
+      <c r="A7" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="53">
+      <c r="B7" s="26">
         <f>INDEX('📋 Детальный реестр'!C27:C32, 1)</f>
         <v/>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="9">
         <f>INDEX('📋 Детальный реестр'!B27:B32, 1)</f>
         <v/>
       </c>
@@ -6403,14 +5650,14 @@
       <c r="J7" s="26" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="57" t="n">
+      <c r="A8" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="54">
+      <c r="B8" s="29">
         <f>INDEX('📋 Детальный реестр'!C33:C38, 1)</f>
         <v/>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="13">
         <f>INDEX('📋 Детальный реестр'!B33:B38, 1)</f>
         <v/>
       </c>
@@ -6439,14 +5686,14 @@
       <c r="J8" s="29" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="56" t="n">
+      <c r="A9" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="26">
         <f>INDEX('📋 Детальный реестр'!C39:C44, 1)</f>
         <v/>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="9">
         <f>INDEX('📋 Детальный реестр'!B39:B44, 1)</f>
         <v/>
       </c>
@@ -6475,14 +5722,14 @@
       <c r="J9" s="26" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="57" t="n">
+      <c r="A10" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="54">
+      <c r="B10" s="29">
         <f>INDEX('📋 Детальный реестр'!C45:C50, 1)</f>
         <v/>
       </c>
-      <c r="C10" s="43">
+      <c r="C10" s="13">
         <f>INDEX('📋 Детальный реестр'!B45:B50, 1)</f>
         <v/>
       </c>
@@ -6511,14 +5758,14 @@
       <c r="J10" s="29" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="56" t="n">
+      <c r="A11" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="53">
+      <c r="B11" s="26">
         <f>INDEX('📋 Детальный реестр'!C51:C56, 1)</f>
         <v/>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="9">
         <f>INDEX('📋 Детальный реестр'!B51:B56, 1)</f>
         <v/>
       </c>
@@ -6547,14 +5794,14 @@
       <c r="J11" s="26" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="57" t="n">
+      <c r="A12" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="54">
+      <c r="B12" s="29">
         <f>INDEX('📋 Детальный реестр'!C57:C62, 1)</f>
         <v/>
       </c>
-      <c r="C12" s="43">
+      <c r="C12" s="13">
         <f>INDEX('📋 Детальный реестр'!B57:B62, 1)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update Vida TikTok metrics to verified 645,952 views (Megahit 245.3k, Superhit 127.7k)
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -5052,10 +5052,10 @@
         <v>0</v>
       </c>
       <c r="I57" s="15" t="n">
-        <v>28526</v>
+        <v>645952</v>
       </c>
       <c r="J57" s="15" t="n">
-        <v>965</v>
+        <v>327</v>
       </c>
       <c r="K57" s="15" t="n">
         <v>0</v>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="Q57" s="15" t="n">
-        <v>985</v>
+        <v>245300</v>
       </c>
       <c r="R57" s="14" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat: update influencer reports with AccountsStats v2 metrics (1.47M views, 236 posts)
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="G8" s="32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8" s="32" t="n">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="G14" s="34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14" s="34" t="n">
         <v>0</v>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>3229</v>
+        <v>3267</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>47</v>
@@ -2276,7 +2276,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="11" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
@@ -2664,7 +2664,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>1511</v>
+        <v>1516</v>
       </c>
       <c r="J21" s="15" t="n">
         <v>52</v>
@@ -3072,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>5326</v>
+        <v>5342</v>
       </c>
       <c r="J27" s="11" t="n">
         <v>179</v>
@@ -3092,7 +3092,7 @@
         <v>0</v>
       </c>
       <c r="O27" s="11" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
@@ -3138,13 +3138,13 @@
         </is>
       </c>
       <c r="G28" s="32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>271</v>
+        <v>377</v>
       </c>
       <c r="J28" s="11" t="n">
         <v>110</v>
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>4385</v>
+        <v>4418</v>
       </c>
       <c r="J33" s="15" t="n">
         <v>44</v>
@@ -3500,7 +3500,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="15" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P33" s="14" t="inlineStr">
         <is>
@@ -3546,13 +3546,13 @@
         </is>
       </c>
       <c r="G34" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H34" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I34" s="15" t="n">
-        <v>1100</v>
+        <v>1398</v>
       </c>
       <c r="J34" s="15" t="n">
         <v>289</v>
@@ -3882,13 +3882,13 @@
         </is>
       </c>
       <c r="G39" s="32" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H39" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>32539</v>
+        <v>32791</v>
       </c>
       <c r="J39" s="11" t="n">
         <v>56</v>
@@ -3908,7 +3908,7 @@
         <v>0</v>
       </c>
       <c r="O39" s="11" t="n">
-        <v>1989</v>
+        <v>2004</v>
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>720296</v>
+        <v>730629</v>
       </c>
       <c r="J40" s="11" t="n">
         <v>9</v>
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="M40" s="11" t="n">
-        <v>782</v>
+        <v>801</v>
       </c>
       <c r="N40" s="22" t="n">
         <v>0</v>
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="G41" s="32" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H41" s="32" t="n">
         <v>0</v>
@@ -4078,13 +4078,13 @@
         </is>
       </c>
       <c r="G42" s="32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H42" s="32" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>3446</v>
+        <v>3459</v>
       </c>
       <c r="J42" s="11" t="n">
         <v>214</v>
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="G44" s="32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H44" s="32" t="n">
         <v>0</v>
@@ -4270,13 +4270,13 @@
         </is>
       </c>
       <c r="G45" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H45" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>2287</v>
+        <v>2564</v>
       </c>
       <c r="J45" s="15" t="n">
         <v>24</v>
@@ -4296,7 +4296,7 @@
         <v>0</v>
       </c>
       <c r="O45" s="15" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="P45" s="14" t="inlineStr">
         <is>
@@ -4338,13 +4338,13 @@
         </is>
       </c>
       <c r="G46" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H46" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I46" s="15" t="n">
-        <v>8411</v>
+        <v>8747</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>271</v>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="M46" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N46" s="23" t="n">
         <v>0</v>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="G47" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H47" s="34" t="n">
         <v>0</v>
@@ -4466,13 +4466,13 @@
         </is>
       </c>
       <c r="G48" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H48" s="34" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="15" t="n">
-        <v>1624</v>
+        <v>1662</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>84</v>
@@ -4594,7 +4594,7 @@
         </is>
       </c>
       <c r="G50" s="34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H50" s="34" t="n">
         <v>0</v>
@@ -4664,7 +4664,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="J51" s="11" t="n">
         <v>320</v>
@@ -4796,7 +4796,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="J53" s="11" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore(dashboard): live metrics update 2026-09-07 14:02:51 (Total views: 1,477,483)
</commit_message>
<xml_diff>
--- a/plitty_influencers_report.xlsx
+++ b/plitty_influencers_report.xlsx
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>3605</v>
+        <v>3606</v>
       </c>
       <c r="J9" s="15" t="n">
         <v>550</v>
@@ -1864,7 +1864,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="15" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P9" s="14" t="inlineStr">
         <is>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>3267</v>
+        <v>3299</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>47</v>
@@ -2276,7 +2276,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="11" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
@@ -2664,7 +2664,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>1516</v>
+        <v>1521</v>
       </c>
       <c r="J21" s="15" t="n">
         <v>52</v>
@@ -3072,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>5342</v>
+        <v>5352</v>
       </c>
       <c r="J27" s="11" t="n">
         <v>179</v>
@@ -3144,7 +3144,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>377</v>
+        <v>436</v>
       </c>
       <c r="J28" s="11" t="n">
         <v>110</v>
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>4418</v>
+        <v>4426</v>
       </c>
       <c r="J33" s="15" t="n">
         <v>44</v>
@@ -3500,7 +3500,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="15" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P33" s="14" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="15" t="n">
-        <v>1398</v>
+        <v>1440</v>
       </c>
       <c r="J34" s="15" t="n">
         <v>289</v>
@@ -3888,7 +3888,7 @@
         <v>0</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>32791</v>
+        <v>33032</v>
       </c>
       <c r="J39" s="11" t="n">
         <v>56</v>
@@ -3908,7 +3908,7 @@
         <v>0</v>
       </c>
       <c r="O39" s="11" t="n">
-        <v>2004</v>
+        <v>2013</v>
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>730629</v>
+        <v>735671</v>
       </c>
       <c r="J40" s="11" t="n">
         <v>9</v>
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="M40" s="11" t="n">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="N40" s="22" t="n">
         <v>0</v>
@@ -4084,7 +4084,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>3459</v>
+        <v>3464</v>
       </c>
       <c r="J42" s="11" t="n">
         <v>214</v>
@@ -4276,7 +4276,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>2564</v>
+        <v>2588</v>
       </c>
       <c r="J45" s="15" t="n">
         <v>24</v>
@@ -4296,7 +4296,7 @@
         <v>0</v>
       </c>
       <c r="O45" s="15" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P45" s="14" t="inlineStr">
         <is>
@@ -4344,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="15" t="n">
-        <v>8747</v>
+        <v>9016</v>
       </c>
       <c r="J46" s="15" t="n">
         <v>271</v>
@@ -4472,7 +4472,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="15" t="n">
-        <v>1662</v>
+        <v>1698</v>
       </c>
       <c r="J48" s="15" t="n">
         <v>84</v>
@@ -4664,7 +4664,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="J51" s="11" t="n">
         <v>320</v>

</xml_diff>